<commit_message>
Also emit the source CSV with a cosine column per model/mode
Alongside the workbook, score_calibration.py writes the calibration CSV back out
unchanged with one cosine column appended per model/mode, keeping the original
column order and row order so it diffs against the input and joins on pair_id.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/calibration_report.xlsx
+++ b/results/calibration_report.xlsx
@@ -534,7 +534,7 @@
         <v>0.9216</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9216</v>
+        <v>0.7474</v>
       </c>
       <c r="I2" t="n">
         <v>0.9223</v>
@@ -578,7 +578,7 @@
         <v>0.6997</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6997</v>
+        <v>0.7423999999999999</v>
       </c>
       <c r="I3" t="n">
         <v>0.7312</v>
@@ -622,7 +622,7 @@
         <v>0.9172</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9172</v>
+        <v>0.8642</v>
       </c>
       <c r="I4" t="n">
         <v>0.8858</v>
@@ -666,7 +666,7 @@
         <v>0.8164</v>
       </c>
       <c r="H5" t="n">
-        <v>0.8164</v>
+        <v>0.6986</v>
       </c>
       <c r="I5" t="n">
         <v>0.7691</v>
@@ -710,7 +710,7 @@
         <v>0.9208</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9208</v>
+        <v>0.749</v>
       </c>
       <c r="I6" t="n">
         <v>0.8144</v>
@@ -754,7 +754,7 @@
         <v>0.8761</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8761</v>
+        <v>0.7179</v>
       </c>
       <c r="I7" t="n">
         <v>0.8248</v>
@@ -798,7 +798,7 @@
         <v>0.7173</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7173</v>
+        <v>0.7204</v>
       </c>
       <c r="I8" t="n">
         <v>0.6819</v>
@@ -842,7 +842,7 @@
         <v>0.6009</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6009</v>
+        <v>0.6403</v>
       </c>
       <c r="I9" t="n">
         <v>0.5570000000000001</v>
@@ -886,7 +886,7 @@
         <v>0.5579</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5579</v>
+        <v>0.5534</v>
       </c>
       <c r="I10" t="n">
         <v>0.6599</v>
@@ -930,7 +930,7 @@
         <v>0.7792</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7792</v>
+        <v>0.7243000000000001</v>
       </c>
       <c r="I11" t="n">
         <v>0.7166</v>
@@ -974,7 +974,7 @@
         <v>0.6938</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6938</v>
+        <v>0.521</v>
       </c>
       <c r="I12" t="n">
         <v>0.7917</v>
@@ -1018,7 +1018,7 @@
         <v>0.6728</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6728</v>
+        <v>0.5772</v>
       </c>
       <c r="I13" t="n">
         <v>0.8183</v>
@@ -1062,7 +1062,7 @@
         <v>0.604</v>
       </c>
       <c r="H14" t="n">
-        <v>0.604</v>
+        <v>0.5954</v>
       </c>
       <c r="I14" t="n">
         <v>0.5628</v>
@@ -1106,7 +1106,7 @@
         <v>0.1053</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1053</v>
+        <v>0.2842</v>
       </c>
       <c r="I15" t="n">
         <v>0.1835</v>
@@ -1150,7 +1150,7 @@
         <v>0.1358</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1358</v>
+        <v>0.1395</v>
       </c>
       <c r="I16" t="n">
         <v>0.2935</v>
@@ -1194,7 +1194,7 @@
         <v>0.2362</v>
       </c>
       <c r="H17" t="n">
-        <v>0.2362</v>
+        <v>0.296</v>
       </c>
       <c r="I17" t="n">
         <v>0.2804</v>
@@ -1238,7 +1238,7 @@
         <v>0.6666</v>
       </c>
       <c r="H18" t="n">
-        <v>0.6666</v>
+        <v>0.6366000000000001</v>
       </c>
       <c r="I18" t="n">
         <v>0.6606</v>
@@ -1282,7 +1282,7 @@
         <v>0.6698</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6698</v>
+        <v>0.6098</v>
       </c>
       <c r="I19" t="n">
         <v>0.6121</v>
@@ -1326,7 +1326,7 @@
         <v>0.594</v>
       </c>
       <c r="H20" t="n">
-        <v>0.594</v>
+        <v>0.6046</v>
       </c>
       <c r="I20" t="n">
         <v>0.5681</v>
@@ -1370,7 +1370,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0.8169</v>
       </c>
       <c r="I21" t="n">
         <v>1</v>
@@ -1446,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0.8169</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -1468,7 +1468,7 @@
         <v>0.8551</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8551</v>
+        <v>0.7603</v>
       </c>
       <c r="E3" t="n">
         <v>0.8246</v>
@@ -1490,7 +1490,7 @@
         <v>0.6435</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6435</v>
+        <v>0.617</v>
       </c>
       <c r="E4" t="n">
         <v>0.6136</v>
@@ -1512,7 +1512,7 @@
         <v>0.7063</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7063</v>
+        <v>0.6713</v>
       </c>
       <c r="E5" t="n">
         <v>0.6879999999999999</v>
@@ -1534,7 +1534,7 @@
         <v>0.6569</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6569</v>
+        <v>0.5645</v>
       </c>
       <c r="E6" t="n">
         <v>0.7243000000000001</v>
@@ -1556,7 +1556,7 @@
         <v>0.1591</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1591</v>
+        <v>0.2399</v>
       </c>
       <c r="E7" t="n">
         <v>0.2525</v>
@@ -1623,7 +1623,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.8169</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -1642,7 +1642,7 @@
         <v>0.8551</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8551</v>
+        <v>0.7603</v>
       </c>
       <c r="D3" t="n">
         <v>0.8246</v>
@@ -1661,7 +1661,7 @@
         <v>0.6435</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6435</v>
+        <v>0.617</v>
       </c>
       <c r="D4" t="n">
         <v>0.6136</v>
@@ -1680,7 +1680,7 @@
         <v>0.7063</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7063</v>
+        <v>0.6713</v>
       </c>
       <c r="D5" t="n">
         <v>0.6879999999999999</v>
@@ -1699,7 +1699,7 @@
         <v>0.6569</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6569</v>
+        <v>0.5645</v>
       </c>
       <c r="D6" t="n">
         <v>0.7243000000000001</v>
@@ -1718,7 +1718,7 @@
         <v>0.1591</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1591</v>
+        <v>0.2399</v>
       </c>
       <c r="D7" t="n">
         <v>0.2525</v>
@@ -1813,7 +1813,7 @@
         <v>0.1489</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1489</v>
+        <v>0.0891</v>
       </c>
       <c r="D12" t="n">
         <v>0.1366</v>
@@ -1832,7 +1832,7 @@
         <v>0.696</v>
       </c>
       <c r="C13" t="n">
-        <v>0.696</v>
+        <v>0.5204</v>
       </c>
       <c r="D13" t="n">
         <v>0.5721000000000001</v>
@@ -1870,7 +1870,7 @@
         <v>0.1053</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1053</v>
+        <v>0.1395</v>
       </c>
       <c r="D15" t="n">
         <v>0.1835</v>
@@ -1889,7 +1889,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>0.8642</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -1908,7 +1908,7 @@
         <v>0.8946</v>
       </c>
       <c r="C17" t="n">
-        <v>0.8946</v>
+        <v>0.7246</v>
       </c>
       <c r="D17" t="n">
         <v>0.8165</v>
@@ -1927,7 +1927,7 @@
         <v>16.638</v>
       </c>
       <c r="C18" t="n">
-        <v>16.638</v>
+        <v>12.2911</v>
       </c>
       <c r="D18" t="n">
         <v>16.7241</v>
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>-0.1741</v>
       </c>
       <c r="D2" t="n">
         <v>-0.195</v>
@@ -2008,7 +2008,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.0426</v>
       </c>
       <c r="D3" t="n">
         <v>-0.166</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>-0.0531</v>
       </c>
       <c r="D4" t="n">
         <v>-0.1362</v>
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>-0.1177</v>
       </c>
       <c r="D5" t="n">
         <v>-0.1027</v>
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>-0.1718</v>
       </c>
       <c r="D6" t="n">
         <v>-0.2192</v>
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>-0.1582</v>
       </c>
       <c r="D7" t="n">
         <v>-0.3513</v>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.0031</v>
       </c>
       <c r="D8" t="n">
         <v>-0.1294</v>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.0394</v>
       </c>
       <c r="D9" t="n">
         <v>-0.098</v>
@@ -2134,7 +2134,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>-0.0045</v>
       </c>
       <c r="D10" t="n">
         <v>-0.196</v>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>-0.0549</v>
       </c>
       <c r="D11" t="n">
         <v>-0.2263</v>
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>-0.1728</v>
       </c>
       <c r="D12" t="n">
         <v>-0.456</v>
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>-0.0956</v>
       </c>
       <c r="D13" t="n">
         <v>-0.3003</v>
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>-0.0086</v>
       </c>
       <c r="D14" t="n">
         <v>-0.1072</v>
@@ -2224,7 +2224,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.1789</v>
       </c>
       <c r="D15" t="n">
         <v>-0.1339</v>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.0038</v>
       </c>
       <c r="D16" t="n">
         <v>-0.18</v>
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.0598</v>
       </c>
       <c r="D17" t="n">
         <v>-0.1173</v>
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>-0.0301</v>
       </c>
       <c r="D18" t="n">
         <v>-0.1599</v>
@@ -2296,7 +2296,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>-0.06</v>
       </c>
       <c r="D19" t="n">
         <v>-0.1544</v>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>0.0105</v>
       </c>
       <c r="D20" t="n">
         <v>-0.1055</v>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>-0.1831</v>
       </c>
       <c r="D21" t="n">
         <v>-0.3052</v>
@@ -2347,7 +2347,7 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>-0.0473</v>
       </c>
       <c r="D23" t="n">
         <v>-0.192</v>

</xml_diff>

<commit_message>
Merge pre-computed 3-large scores into the calibration report
--extra label=path.csv pulls pair_id,cosine columns from a file scored
elsewhere, defaulting to data/results_detail_v1_pairs.csv as text3large. Rows
outside the calibration set are ignored, which skips that file's trailing
=== SUMMARY === block, and where the file carries text_a/text_b they are checked
against the calibration file so a score cannot be attached to a pair it was not
computed on. Tier stats are nan-safe for a column missing some pairs.

The per-mode workbooks are gone; calibration_report.xlsx already carries every
mode as its own column, and calibration_report.csv is the source CSV with one
cosine column appended per model/mode.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/calibration_report.xlsx
+++ b/results/calibration_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,6 +499,11 @@
           <t>vn_embedding/instruct</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>text3large</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -542,6 +548,9 @@
       <c r="J2" t="n">
         <v>0.7272999999999999</v>
       </c>
+      <c r="K2" t="n">
+        <v>0.8629</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -586,6 +595,9 @@
       <c r="J3" t="n">
         <v>0.5652</v>
       </c>
+      <c r="K3" t="n">
+        <v>0.7864</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -630,6 +642,9 @@
       <c r="J4" t="n">
         <v>0.7497</v>
       </c>
+      <c r="K4" t="n">
+        <v>0.9396</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -674,6 +689,9 @@
       <c r="J5" t="n">
         <v>0.6664</v>
       </c>
+      <c r="K5" t="n">
+        <v>0.8532</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -718,6 +736,9 @@
       <c r="J6" t="n">
         <v>0.5952</v>
       </c>
+      <c r="K6" t="n">
+        <v>0.8416</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -762,6 +783,9 @@
       <c r="J7" t="n">
         <v>0.4735</v>
       </c>
+      <c r="K7" t="n">
+        <v>0.8665</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -806,6 +830,9 @@
       <c r="J8" t="n">
         <v>0.5525</v>
       </c>
+      <c r="K8" t="n">
+        <v>0.631</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -850,6 +877,9 @@
       <c r="J9" t="n">
         <v>0.459</v>
       </c>
+      <c r="K9" t="n">
+        <v>0.5709</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -894,6 +924,9 @@
       <c r="J10" t="n">
         <v>0.4639</v>
       </c>
+      <c r="K10" t="n">
+        <v>0.6024</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -938,6 +971,9 @@
       <c r="J11" t="n">
         <v>0.4903</v>
       </c>
+      <c r="K11" t="n">
+        <v>0.7012</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -982,6 +1018,9 @@
       <c r="J12" t="n">
         <v>0.3357</v>
       </c>
+      <c r="K12" t="n">
+        <v>0.8915999999999999</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1026,6 +1065,9 @@
       <c r="J13" t="n">
         <v>0.518</v>
       </c>
+      <c r="K13" t="n">
+        <v>0.7647</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1070,6 +1112,9 @@
       <c r="J14" t="n">
         <v>0.4557</v>
       </c>
+      <c r="K14" t="n">
+        <v>0.5758</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1114,6 +1159,9 @@
       <c r="J15" t="n">
         <v>0.0496</v>
       </c>
+      <c r="K15" t="n">
+        <v>0.2803</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1158,6 +1206,9 @@
       <c r="J16" t="n">
         <v>0.1135</v>
       </c>
+      <c r="K16" t="n">
+        <v>0.3041</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1202,6 +1253,9 @@
       <c r="J17" t="n">
         <v>0.1631</v>
       </c>
+      <c r="K17" t="n">
+        <v>0.3269</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1246,6 +1300,9 @@
       <c r="J18" t="n">
         <v>0.5007</v>
       </c>
+      <c r="K18" t="n">
+        <v>0.7192</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1290,6 +1347,9 @@
       <c r="J19" t="n">
         <v>0.4577</v>
       </c>
+      <c r="K19" t="n">
+        <v>0.5534</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1334,6 +1394,9 @@
       <c r="J20" t="n">
         <v>0.4626</v>
       </c>
+      <c r="K20" t="n">
+        <v>0.6137</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1377,6 +1440,9 @@
       </c>
       <c r="J21" t="n">
         <v>0.6948</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1390,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -1399,6 +1465,7 @@
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1432,6 +1499,11 @@
           <t>vn_embedding/instruct</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>text3large</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1454,6 +1526,9 @@
       <c r="F2" t="n">
         <v>0.6948</v>
       </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1476,6 +1551,9 @@
       <c r="F3" t="n">
         <v>0.6608000000000001</v>
       </c>
+      <c r="G3" t="n">
+        <v>0.8567</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1498,6 +1576,9 @@
       <c r="F4" t="n">
         <v>0.4737</v>
       </c>
+      <c r="G4" t="n">
+        <v>0.6288</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1520,6 +1601,9 @@
       <c r="F5" t="n">
         <v>0.4878</v>
       </c>
+      <c r="G5" t="n">
+        <v>0.6744</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1542,6 +1626,9 @@
       <c r="F6" t="n">
         <v>0.4364</v>
       </c>
+      <c r="G6" t="n">
+        <v>0.744</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1563,6 +1650,9 @@
       </c>
       <c r="F7" t="n">
         <v>0.1087</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.3038</v>
       </c>
     </row>
   </sheetData>
@@ -1576,7 +1666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -1584,6 +1674,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1612,6 +1703,11 @@
           <t>vn_embedding/instruct</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>text3large</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1631,6 +1727,9 @@
       <c r="E2" t="n">
         <v>0.6948</v>
       </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1650,6 +1749,9 @@
       <c r="E3" t="n">
         <v>0.6608000000000001</v>
       </c>
+      <c r="F3" t="n">
+        <v>0.8567</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1669,6 +1771,9 @@
       <c r="E4" t="n">
         <v>0.4737</v>
       </c>
+      <c r="F4" t="n">
+        <v>0.6288</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1688,6 +1793,9 @@
       <c r="E5" t="n">
         <v>0.4878</v>
       </c>
+      <c r="F5" t="n">
+        <v>0.6744</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1707,6 +1815,9 @@
       <c r="E6" t="n">
         <v>0.4364</v>
       </c>
+      <c r="F6" t="n">
+        <v>0.744</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1726,6 +1837,9 @@
       <c r="E7" t="n">
         <v>0.1087</v>
       </c>
+      <c r="F7" t="n">
+        <v>0.3038</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1745,6 +1859,9 @@
       <c r="E8" t="b">
         <v>1</v>
       </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1764,6 +1881,9 @@
       <c r="E9" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="F9" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1783,6 +1903,9 @@
       <c r="E10" t="b">
         <v>1</v>
       </c>
+      <c r="F10" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1802,6 +1925,9 @@
       <c r="E11" t="b">
         <v>1</v>
       </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1821,6 +1947,9 @@
       <c r="E12" t="n">
         <v>0.1729</v>
       </c>
+      <c r="F12" t="n">
+        <v>0.1823</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1840,6 +1969,9 @@
       <c r="E13" t="n">
         <v>0.552</v>
       </c>
+      <c r="F13" t="n">
+        <v>0.553</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1859,6 +1991,9 @@
       <c r="E14" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="F14" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1878,6 +2013,9 @@
       <c r="E15" t="n">
         <v>0.0496</v>
       </c>
+      <c r="F15" t="n">
+        <v>0.2803</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1897,6 +2035,9 @@
       <c r="E16" t="n">
         <v>0.7497</v>
       </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1916,6 +2057,9 @@
       <c r="E17" t="n">
         <v>0.7000999999999999</v>
       </c>
+      <c r="F17" t="n">
+        <v>0.7197</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1934,6 +2078,9 @@
       </c>
       <c r="E18" t="n">
         <v>24.7024</v>
+      </c>
+      <c r="F18" t="n">
+        <v>25.3356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Write up the calibration results
All six configurations now read T0 = 1.000, confirming the symmetric fix. Adds
--exclude, defaulting to vn_embedding/instruct, since that model defines no
instruction and any vectors still on disk under that name are from a superseded run.

Headline findings, in results/calibration_summary.md: every model including
text3large fails the vocabulary-gap rung, so a differently-worded correct passage
ranks below a same-document wrong-attribute one; text3large separates T1 from T2
best; vn_embedding and text3large both fail to tell two documents apart while both
Qwen models pass; and the instruction prefix compresses the cosine range without
repairing any rung.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/calibration_report.xlsx
+++ b/results/calibration_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -443,9 +443,10 @@
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,15 +492,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>qwen3_vl_2b/no_instruct</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>qwen3_vl_2b/instruct</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>vn_embedding/no_instruct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>vn_embedding/instruct</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>text3large</t>
         </is>
@@ -537,18 +543,21 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.9216</v>
+        <v>0.9215</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7474</v>
+        <v>0.9445</v>
       </c>
       <c r="I2" t="n">
+        <v>0.9339</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.9530999999999999</v>
+      </c>
+      <c r="K2" t="n">
         <v>0.9223</v>
       </c>
-      <c r="J2" t="n">
-        <v>0.7272999999999999</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.8629</v>
       </c>
     </row>
@@ -584,18 +593,21 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.6997</v>
+        <v>0.6998</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7423999999999999</v>
+        <v>0.821</v>
       </c>
       <c r="I3" t="n">
+        <v>0.7714</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="K3" t="n">
         <v>0.7312</v>
       </c>
-      <c r="J3" t="n">
-        <v>0.5652</v>
-      </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.7864</v>
       </c>
     </row>
@@ -634,15 +646,18 @@
         <v>0.9172</v>
       </c>
       <c r="H4" t="n">
-        <v>0.8642</v>
+        <v>0.9567</v>
       </c>
       <c r="I4" t="n">
+        <v>0.9272</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9397</v>
+      </c>
+      <c r="K4" t="n">
         <v>0.8858</v>
       </c>
-      <c r="J4" t="n">
-        <v>0.7497</v>
-      </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.9396</v>
       </c>
     </row>
@@ -678,18 +693,21 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.8164</v>
+        <v>0.8165</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6986</v>
+        <v>0.9328</v>
       </c>
       <c r="I5" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.9367</v>
+      </c>
+      <c r="K5" t="n">
         <v>0.7691</v>
       </c>
-      <c r="J5" t="n">
-        <v>0.6664</v>
-      </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.8532</v>
       </c>
     </row>
@@ -725,18 +743,21 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.9208</v>
+        <v>0.9207</v>
       </c>
       <c r="H6" t="n">
-        <v>0.749</v>
+        <v>0.9671999999999999</v>
       </c>
       <c r="I6" t="n">
+        <v>0.9326</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.9498</v>
+      </c>
+      <c r="K6" t="n">
         <v>0.8144</v>
       </c>
-      <c r="J6" t="n">
-        <v>0.5952</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.8416</v>
       </c>
     </row>
@@ -772,18 +793,21 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.8761</v>
+        <v>0.8764999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7179</v>
+        <v>0.9766</v>
       </c>
       <c r="I7" t="n">
+        <v>0.8715000000000001</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.9403</v>
+      </c>
+      <c r="K7" t="n">
         <v>0.8248</v>
       </c>
-      <c r="J7" t="n">
-        <v>0.4735</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.8665</v>
       </c>
     </row>
@@ -819,18 +843,21 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.7173</v>
+        <v>0.7171999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7204</v>
+        <v>0.8346</v>
       </c>
       <c r="I8" t="n">
+        <v>0.6214</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.7379</v>
+      </c>
+      <c r="K8" t="n">
         <v>0.6819</v>
       </c>
-      <c r="J8" t="n">
-        <v>0.5525</v>
-      </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.631</v>
       </c>
     </row>
@@ -866,18 +893,21 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.6009</v>
+        <v>0.6008</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6403</v>
+        <v>0.7486</v>
       </c>
       <c r="I9" t="n">
+        <v>0.6741</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.7302</v>
+      </c>
+      <c r="K9" t="n">
         <v>0.5570000000000001</v>
       </c>
-      <c r="J9" t="n">
-        <v>0.459</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.5709</v>
       </c>
     </row>
@@ -913,18 +943,21 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.5579</v>
+        <v>0.5581</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5534</v>
+        <v>0.7671</v>
       </c>
       <c r="I10" t="n">
+        <v>0.7719</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.7743</v>
+      </c>
+      <c r="K10" t="n">
         <v>0.6599</v>
       </c>
-      <c r="J10" t="n">
-        <v>0.4639</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>0.6024</v>
       </c>
     </row>
@@ -960,18 +993,21 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.7792</v>
+        <v>0.7793</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7243000000000001</v>
+        <v>0.7939000000000001</v>
       </c>
       <c r="I11" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="K11" t="n">
         <v>0.7166</v>
       </c>
-      <c r="J11" t="n">
-        <v>0.4903</v>
-      </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>0.7012</v>
       </c>
     </row>
@@ -1007,18 +1043,21 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.6938</v>
+        <v>0.6935</v>
       </c>
       <c r="H12" t="n">
-        <v>0.521</v>
+        <v>0.7241</v>
       </c>
       <c r="I12" t="n">
+        <v>0.8247</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.8374</v>
+      </c>
+      <c r="K12" t="n">
         <v>0.7917</v>
       </c>
-      <c r="J12" t="n">
-        <v>0.3357</v>
-      </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>0.8915999999999999</v>
       </c>
     </row>
@@ -1054,18 +1093,21 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.6728</v>
+        <v>0.6727</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5772</v>
+        <v>0.6266</v>
       </c>
       <c r="I13" t="n">
+        <v>0.7348</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.6246</v>
+      </c>
+      <c r="K13" t="n">
         <v>0.8183</v>
       </c>
-      <c r="J13" t="n">
-        <v>0.518</v>
-      </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.7647</v>
       </c>
     </row>
@@ -1101,18 +1143,21 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.604</v>
+        <v>0.6039</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5954</v>
+        <v>0.7231</v>
       </c>
       <c r="I14" t="n">
+        <v>0.6711</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.6942</v>
+      </c>
+      <c r="K14" t="n">
         <v>0.5628</v>
       </c>
-      <c r="J14" t="n">
-        <v>0.4557</v>
-      </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>0.5758</v>
       </c>
     </row>
@@ -1148,18 +1193,21 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.1053</v>
+        <v>0.1054</v>
       </c>
       <c r="H15" t="n">
-        <v>0.2842</v>
+        <v>0.4203</v>
       </c>
       <c r="I15" t="n">
+        <v>0.1677</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.4358</v>
+      </c>
+      <c r="K15" t="n">
         <v>0.1835</v>
       </c>
-      <c r="J15" t="n">
-        <v>0.0496</v>
-      </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>0.2803</v>
       </c>
     </row>
@@ -1198,15 +1246,18 @@
         <v>0.1358</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1395</v>
+        <v>0.385</v>
       </c>
       <c r="I16" t="n">
+        <v>0.2894</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.3834</v>
+      </c>
+      <c r="K16" t="n">
         <v>0.2935</v>
       </c>
-      <c r="J16" t="n">
-        <v>0.1135</v>
-      </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>0.3041</v>
       </c>
     </row>
@@ -1242,18 +1293,21 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.2362</v>
+        <v>0.2364</v>
       </c>
       <c r="H17" t="n">
-        <v>0.296</v>
+        <v>0.4135</v>
       </c>
       <c r="I17" t="n">
+        <v>0.4207</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.3849</v>
+      </c>
+      <c r="K17" t="n">
         <v>0.2804</v>
       </c>
-      <c r="J17" t="n">
-        <v>0.1631</v>
-      </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>0.3269</v>
       </c>
     </row>
@@ -1289,18 +1343,21 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.6666</v>
+        <v>0.6667</v>
       </c>
       <c r="H18" t="n">
-        <v>0.6366000000000001</v>
+        <v>0.7266</v>
       </c>
       <c r="I18" t="n">
+        <v>0.7288</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.6942</v>
+      </c>
+      <c r="K18" t="n">
         <v>0.6606</v>
       </c>
-      <c r="J18" t="n">
-        <v>0.5007</v>
-      </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>0.7192</v>
       </c>
     </row>
@@ -1339,15 +1396,18 @@
         <v>0.6698</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6098</v>
+        <v>0.7375</v>
       </c>
       <c r="I19" t="n">
+        <v>0.7637</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.6793</v>
+      </c>
+      <c r="K19" t="n">
         <v>0.6121</v>
       </c>
-      <c r="J19" t="n">
-        <v>0.4577</v>
-      </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>0.5534</v>
       </c>
     </row>
@@ -1383,18 +1443,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.594</v>
+        <v>0.5938</v>
       </c>
       <c r="H20" t="n">
-        <v>0.6046</v>
+        <v>0.7119</v>
       </c>
       <c r="I20" t="n">
+        <v>0.7183</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="K20" t="n">
         <v>0.5681</v>
       </c>
-      <c r="J20" t="n">
-        <v>0.4626</v>
-      </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>0.6137</v>
       </c>
     </row>
@@ -1433,15 +1496,18 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>0.8169</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>0.6948</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1456,16 +1522,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
     <col width="3" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1491,15 +1558,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>qwen3_vl_2b/no_instruct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>qwen3_vl_2b/instruct</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>vn_embedding/no_instruct</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>vn_embedding/instruct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>text3large</t>
         </is>
@@ -1518,15 +1590,18 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8169</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6948</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1543,15 +1618,18 @@
         <v>0.8551</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7603</v>
+        <v>0.9244</v>
       </c>
       <c r="E3" t="n">
+        <v>0.8858</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9186</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.8246</v>
       </c>
-      <c r="F3" t="n">
-        <v>0.6608000000000001</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.8567</v>
       </c>
     </row>
@@ -1565,18 +1643,21 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6435</v>
+        <v>0.6434</v>
       </c>
       <c r="D4" t="n">
-        <v>0.617</v>
+        <v>0.7252999999999999</v>
       </c>
       <c r="E4" t="n">
+        <v>0.7369</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.6715</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.6136</v>
       </c>
-      <c r="F4" t="n">
-        <v>0.4737</v>
-      </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.6288</v>
       </c>
     </row>
@@ -1590,18 +1671,21 @@
         <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7063</v>
+        <v>0.7064</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6713</v>
+        <v>0.8242</v>
       </c>
       <c r="E5" t="n">
+        <v>0.7452</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.7873</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.6879999999999999</v>
       </c>
-      <c r="F5" t="n">
-        <v>0.4878</v>
-      </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.6744</v>
       </c>
     </row>
@@ -1615,18 +1699,21 @@
         <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6569</v>
+        <v>0.6567</v>
       </c>
       <c r="D6" t="n">
-        <v>0.5645</v>
+        <v>0.6913</v>
       </c>
       <c r="E6" t="n">
+        <v>0.7435</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.7243000000000001</v>
       </c>
-      <c r="F6" t="n">
-        <v>0.4364</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>0.744</v>
       </c>
     </row>
@@ -1640,18 +1727,21 @@
         <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1591</v>
+        <v>0.1592</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2399</v>
+        <v>0.4063</v>
       </c>
       <c r="E7" t="n">
+        <v>0.2926</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4014</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.2525</v>
       </c>
-      <c r="F7" t="n">
-        <v>0.1087</v>
-      </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0.3038</v>
       </c>
     </row>
@@ -1666,15 +1756,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1695,15 +1786,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>qwen3_vl_2b/no_instruct</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>qwen3_vl_2b/instruct</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>vn_embedding/no_instruct</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>vn_embedding/instruct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>text3large</t>
         </is>
@@ -1719,15 +1815,18 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8169</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6948</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1741,15 +1840,18 @@
         <v>0.8551</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7603</v>
+        <v>0.9244</v>
       </c>
       <c r="D3" t="n">
+        <v>0.8858</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.9186</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.8246</v>
       </c>
-      <c r="E3" t="n">
-        <v>0.6608000000000001</v>
-      </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.8567</v>
       </c>
     </row>
@@ -1760,18 +1862,21 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6435</v>
+        <v>0.6434</v>
       </c>
       <c r="C4" t="n">
-        <v>0.617</v>
+        <v>0.7252999999999999</v>
       </c>
       <c r="D4" t="n">
+        <v>0.7369</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6715</v>
+      </c>
+      <c r="F4" t="n">
         <v>0.6136</v>
       </c>
-      <c r="E4" t="n">
-        <v>0.4737</v>
-      </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.6288</v>
       </c>
     </row>
@@ -1782,18 +1887,21 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7063</v>
+        <v>0.7064</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6713</v>
+        <v>0.8242</v>
       </c>
       <c r="D5" t="n">
+        <v>0.7452</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7873</v>
+      </c>
+      <c r="F5" t="n">
         <v>0.6879999999999999</v>
       </c>
-      <c r="E5" t="n">
-        <v>0.4878</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0.6744</v>
       </c>
     </row>
@@ -1804,18 +1912,21 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.6569</v>
+        <v>0.6567</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5645</v>
+        <v>0.6913</v>
       </c>
       <c r="D6" t="n">
+        <v>0.7435</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="F6" t="n">
         <v>0.7243000000000001</v>
       </c>
-      <c r="E6" t="n">
-        <v>0.4364</v>
-      </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>0.744</v>
       </c>
     </row>
@@ -1826,18 +1937,21 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1591</v>
+        <v>0.1592</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2399</v>
+        <v>0.4063</v>
       </c>
       <c r="D7" t="n">
+        <v>0.2926</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.4014</v>
+      </c>
+      <c r="F7" t="n">
         <v>0.2525</v>
       </c>
-      <c r="E7" t="n">
-        <v>0.1087</v>
-      </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>0.3038</v>
       </c>
     </row>
@@ -1862,6 +1976,9 @@
       <c r="F8" t="b">
         <v>1</v>
       </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1884,6 +2001,9 @@
       <c r="F9" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="G9" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1897,8 +2017,8 @@
       <c r="C10" t="b">
         <v>1</v>
       </c>
-      <c r="D10" s="2" t="b">
-        <v>0</v>
+      <c r="D10" t="b">
+        <v>1</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -1906,6 +2026,9 @@
       <c r="F10" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="G10" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1928,6 +2051,9 @@
       <c r="F11" t="b">
         <v>1</v>
       </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1936,18 +2062,21 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1489</v>
+        <v>0.1487</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0891</v>
+        <v>0.1003</v>
       </c>
       <c r="D12" t="n">
+        <v>0.1406</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1313</v>
+      </c>
+      <c r="F12" t="n">
         <v>0.1366</v>
       </c>
-      <c r="E12" t="n">
-        <v>0.1729</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>0.1823</v>
       </c>
     </row>
@@ -1958,18 +2087,21 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.696</v>
+        <v>0.6959</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5204</v>
+        <v>0.5182</v>
       </c>
       <c r="D13" t="n">
+        <v>0.5931999999999999</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.5173</v>
+      </c>
+      <c r="F13" t="n">
         <v>0.5721000000000001</v>
       </c>
-      <c r="E13" t="n">
-        <v>0.552</v>
-      </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>0.553</v>
       </c>
     </row>
@@ -1994,6 +2126,9 @@
       <c r="F14" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="G14" s="2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2002,18 +2137,21 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1053</v>
+        <v>0.1054</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1395</v>
+        <v>0.385</v>
       </c>
       <c r="D15" t="n">
+        <v>0.1677</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.3834</v>
+      </c>
+      <c r="F15" t="n">
         <v>0.1835</v>
       </c>
-      <c r="E15" t="n">
-        <v>0.0496</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>0.2803</v>
       </c>
     </row>
@@ -2027,15 +2165,18 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8642</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>0.7497</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2049,15 +2190,18 @@
         <v>0.8946</v>
       </c>
       <c r="C17" t="n">
-        <v>0.7246</v>
+        <v>0.615</v>
       </c>
       <c r="D17" t="n">
+        <v>0.8323</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.6166</v>
+      </c>
+      <c r="F17" t="n">
         <v>0.8165</v>
       </c>
-      <c r="E17" t="n">
-        <v>0.7000999999999999</v>
-      </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>0.7197</v>
       </c>
     </row>
@@ -2068,18 +2212,21 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>16.638</v>
+        <v>16.6266</v>
       </c>
       <c r="C18" t="n">
-        <v>12.2911</v>
+        <v>16.3061</v>
       </c>
       <c r="D18" t="n">
+        <v>16.8931</v>
+      </c>
+      <c r="E18" t="n">
+        <v>21.2973</v>
+      </c>
+      <c r="F18" t="n">
         <v>16.7241</v>
       </c>
-      <c r="E18" t="n">
-        <v>24.7024</v>
-      </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>25.3356</v>
       </c>
     </row>
@@ -2100,7 +2247,7 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2121,7 +2268,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>vn_embedding: instruct - no_instruct</t>
+          <t>qwen3_vl_2b: instruct - no_instruct</t>
         </is>
       </c>
     </row>
@@ -2137,10 +2284,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.1741</v>
+        <v>0.023</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.195</v>
+        <v>0.0192</v>
       </c>
     </row>
     <row r="3">
@@ -2155,10 +2302,10 @@
         </is>
       </c>
       <c r="C3" t="n">
+        <v>0.1212</v>
+      </c>
+      <c r="D3" t="n">
         <v>0.0426</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-0.166</v>
       </c>
     </row>
     <row r="4">
@@ -2173,10 +2320,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.0531</v>
+        <v>0.0395</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.1362</v>
+        <v>0.0125</v>
       </c>
     </row>
     <row r="5">
@@ -2191,10 +2338,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.1177</v>
+        <v>0.1163</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1027</v>
+        <v>0.0727</v>
       </c>
     </row>
     <row r="6">
@@ -2209,10 +2356,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.1718</v>
+        <v>0.0465</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.2192</v>
+        <v>0.0172</v>
       </c>
     </row>
     <row r="7">
@@ -2227,10 +2374,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.1582</v>
+        <v>0.1001</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.3513</v>
+        <v>0.0687</v>
       </c>
     </row>
     <row r="8">
@@ -2245,10 +2392,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0031</v>
+        <v>0.1174</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.1294</v>
+        <v>0.1165</v>
       </c>
     </row>
     <row r="9">
@@ -2263,10 +2410,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0394</v>
+        <v>0.1478</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.098</v>
+        <v>0.0561</v>
       </c>
     </row>
     <row r="10">
@@ -2281,10 +2428,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.0045</v>
+        <v>0.2091</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.196</v>
+        <v>0.0023</v>
       </c>
     </row>
     <row r="11">
@@ -2299,10 +2446,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.0549</v>
+        <v>0.0146</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.2263</v>
+        <v>-0.033</v>
       </c>
     </row>
     <row r="12">
@@ -2317,10 +2464,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.1728</v>
+        <v>0.0306</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.456</v>
+        <v>0.0127</v>
       </c>
     </row>
     <row r="13">
@@ -2335,10 +2482,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.0956</v>
+        <v>-0.0461</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.3003</v>
+        <v>-0.1102</v>
       </c>
     </row>
     <row r="14">
@@ -2353,10 +2500,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.0086</v>
+        <v>0.1192</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.1072</v>
+        <v>0.0231</v>
       </c>
     </row>
     <row r="15">
@@ -2371,10 +2518,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.1789</v>
+        <v>0.3149</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.1339</v>
+        <v>0.2681</v>
       </c>
     </row>
     <row r="16">
@@ -2389,10 +2536,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.0038</v>
+        <v>0.2493</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.18</v>
+        <v>0.094</v>
       </c>
     </row>
     <row r="17">
@@ -2407,10 +2554,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.0598</v>
+        <v>0.1771</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1173</v>
+        <v>-0.0358</v>
       </c>
     </row>
     <row r="18">
@@ -2425,10 +2572,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-0.0301</v>
+        <v>0.0599</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.1599</v>
+        <v>-0.0345</v>
       </c>
     </row>
     <row r="19">
@@ -2443,10 +2590,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-0.06</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1544</v>
+        <v>-0.0844</v>
       </c>
     </row>
     <row r="20">
@@ -2461,10 +2608,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.0105</v>
+        <v>0.1181</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1055</v>
+        <v>-0.0772</v>
       </c>
     </row>
     <row r="21">
@@ -2479,10 +2626,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-0.1831</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.3052</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="22"/>
@@ -2494,10 +2641,10 @@
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="n">
-        <v>-0.0473</v>
+        <v>0.1013</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.192</v>
+        <v>0.0215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>